<commit_message>
respaldo automático 2026-07-24 15:57:51
</commit_message>
<xml_diff>
--- a/nexus/conector-tek/data/masivas/masiva-masiva.xlsx
+++ b/nexus/conector-tek/data/masivas/masiva-masiva.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Cuenta origen (obligatorio)</t>
   </si>
@@ -58,19 +58,25 @@
     <t>CLP</t>
   </si>
   <si>
-    <t>123</t>
+    <t>19800476890</t>
+  </si>
+  <si>
+    <t>051</t>
+  </si>
+  <si>
+    <t>196892281</t>
+  </si>
+  <si>
+    <t>JOAQUIN ELIAS MALUK</t>
+  </si>
+  <si>
+    <t>prueba masiva</t>
+  </si>
+  <si>
+    <t>joaquin.maluk@gmail.com</t>
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>ANA CLARA SPA</t>
   </si>
 </sst>
 </file>
@@ -521,19 +527,19 @@
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="K2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="L2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
respaldo automático 2026-07-25 00:13:39
</commit_message>
<xml_diff>
--- a/nexus/conector-tek/data/masivas/masiva-masiva.xlsx
+++ b/nexus/conector-tek/data/masivas/masiva-masiva.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>Cuenta origen (obligatorio)</t>
   </si>
@@ -58,25 +58,22 @@
     <t>CLP</t>
   </si>
   <si>
-    <t>19800476890</t>
-  </si>
-  <si>
-    <t>051</t>
-  </si>
-  <si>
-    <t>196892281</t>
-  </si>
-  <si>
-    <t>JOAQUIN ELIAS MALUK</t>
-  </si>
-  <si>
-    <t>prueba masiva</t>
-  </si>
-  <si>
-    <t>joaquin.maluk@gmail.com</t>
+    <t>72019474</t>
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>761066366</t>
+  </si>
+  <si>
+    <t>IMPORTADORA HN SPA</t>
+  </si>
+  <si>
+    <t>Devolución préstamo</t>
+  </si>
+  <si>
+    <t>ANA CLARA SPA</t>
   </si>
 </sst>
 </file>
@@ -454,7 +451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="8" max="8" width="9" style="1" customWidth="1"/>
@@ -524,13 +521,13 @@
         <v>18</v>
       </c>
       <c r="H2" s="1">
-        <v>1</v>
+        <v>7000000</v>
       </c>
       <c r="I2" t="s">
         <v>19</v>
       </c>
       <c r="J2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="K2" t="s">
         <v>19</v>
@@ -539,7 +536,48 @@
         <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>21</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="1">
+        <v>3000000</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M3" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>